<commit_message>
Add LOINC code column to review export
Each SNOMED-LOINC observable carries its LOINC code as an RF2 alternate
identifier (sct2_Identifier, scheme 30051010000102) inside the LOINCSNOMED
edition itself — Snowstorm does not expose it via API, so review_export.py
reads the extracted Identifier file (1:1 map, 45014 entries). LOINC is now the
leading column in every XLSX/CSV. Coverage 977/987 (missing = panels / target
values / abstract groupers without a LOINC code). Raw RF2 extract is
gitignored as a licensed release artifact.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/review/local-2026-03-21/hba1c_review.xlsx
+++ b/output/review/local-2026-03-21/hba1c_review.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hba1c" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'hba1c'!$A$12:$K$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'hba1c'!$A$12:$L$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,20 +443,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -592,59 +593,65 @@
       <c r="I12" s="1" t="n"/>
       <c r="J12" s="1" t="n"/>
       <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>LOINC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>SCTID</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>FSN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>PT</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Complete aggregation</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Quantitative (all numeric)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Quantitative &amp; convertible</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Qualitative (ordinal / nominal / presence)</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Semi-quantitative (test strip)</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Panel / order code (no Property)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Use case</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
@@ -653,32 +660,32 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>4548-4</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
           <t>558301010000102</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Mass fraction of glycated hemoglobin-A1c to hemoglobin.total in blood at point in time (observable entity)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total in Blood</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -696,12 +703,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
@@ -710,32 +722,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>17855-8</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
           <t>501091010000106</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Mass fraction of glycated hemoglobin-A1c to hemoglobin.total in blood at point in time by calculation (observable entity)</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total in Blood by calculation</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -753,12 +765,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
@@ -767,32 +784,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>4549-2</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>558311010000104</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Mass fraction of glycated hemoglobin-A1c to hemoglobin.total in blood at point in time by electrophoresis (observable entity)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total in Blood by Electrophoresis</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -810,12 +827,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
@@ -824,32 +846,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>17856-6</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>501101010000102</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Mass fraction of glycated hemoglobin-A1c to hemoglobin.total in blood at point in time by high pressure liquid chromatography (observable entity)</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total in Blood by HPLC</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -867,12 +889,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
@@ -881,32 +908,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>62388-4</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
           <t>602671010000102</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Mass fraction of glycated hemoglobin-A1c to hemoglobin.total in blood at point in time by JDS/JSCC (observable entity)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total in Blood by JDS/JSCC protocol</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -924,12 +951,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
@@ -938,32 +970,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>96595-4</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
           <t>623431010000103</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Mass fraction of glycated hemoglobin-A1c to hemoglobin.total in dried blood spot at point in time (observable entity)</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total in DBS</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -981,12 +1013,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
@@ -995,32 +1032,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>59261-8</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
           <t>598941010000105</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Substance fraction of glycated hemoglobin-A1c standardized per IFCC-RMP for CDT to hemoglobin.total in blood at point in time (observable entity)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c/Hemoglobin.total standardized per IFCC-RMP for CDT in Blood</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1038,38 +1075,39 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>quantitative</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>408591000</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c target (observable entity)</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>HBA1c target</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1080,9 +1118,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1095,38 +1133,39 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>quantitative_convertible</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Measurement property, no scale asserted (generic) + concentration property</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>446074002</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c target value using International Federation of Clinical Chemistry and Laboratory Medicine standardized method (observable entity)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c target value using International Federation of Clinical Chemistry and Laboratory Medicine standardized method</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1137,9 +1176,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1152,12 +1191,17 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>quantitative_convertible</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Measurement property, no scale asserted (generic) + concentration property</t>
         </is>
@@ -1166,24 +1210,24 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>41995-2</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
           <t>43401010000104</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Mass concentration of glycated hemoglobin-A1c in blood at point in time (observable entity)</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Hemoglobin A1c [Mass/volume] in Blood</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1194,9 +1238,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1209,19 +1253,24 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>quantitative_convertible</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Quantitative scale + concentration property</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A12:K23"/>
+  <autoFilter ref="A12:L23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>